<commit_message>
Add empty New Section to project proposal
</commit_message>
<xml_diff>
--- a/docs/diagrams/base-enterprise.xlsx
+++ b/docs/diagrams/base-enterprise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stolle\git\frank1stolle-blip\OFTP2OnboardingService\docs\diagrams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E8D1C82-83BF-416D-A7B7-94DB7C7A5E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{135BCBE5-B0C2-4D9C-91C2-9BE05112915F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="4575" windowWidth="28680" windowHeight="14970" xr2:uid="{3E93D1C4-9B1F-4A0A-95BF-AEED9CDE6346}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Onboardings included</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>iPaaS / on-premises instance</t>
+  </si>
+  <si>
+    <t>External API Integration</t>
   </si>
 </sst>
 </file>
@@ -123,17 +126,17 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>480855</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>59325</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>564015</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>141045</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="4" name="Freihand 3">
@@ -152,7 +155,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="4" name="Freihand 3">
@@ -188,17 +191,17 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>480855</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>49800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>564015</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>131520</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="5" name="Freihand 4">
@@ -217,7 +220,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="5" name="Freihand 4">
@@ -262,8 +265,8 @@
       <xdr:row>5</xdr:row>
       <xdr:rowOff>131520</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="6" name="Freihand 5">
@@ -282,7 +285,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="6" name="Freihand 5">
@@ -327,8 +330,8 @@
       <xdr:row>5</xdr:row>
       <xdr:rowOff>145808</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="7" name="Freihand 6">
@@ -347,7 +350,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="7" name="Freihand 6">
@@ -392,8 +395,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>141045</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="8" name="Freihand 7">
@@ -412,7 +415,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="8" name="Freihand 7">
@@ -448,17 +451,17 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>461602</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>85575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>512002</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>85935</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="15" name="Freihand 14">
@@ -477,7 +480,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="15" name="Freihand 14">
@@ -522,8 +525,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>109747</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="16" name="Freihand 15">
@@ -542,7 +545,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="16" name="Freihand 15">
@@ -578,17 +581,17 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>461602</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>85575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>512002</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>85935</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="17" name="Freihand 16">
@@ -607,7 +610,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="17" name="Freihand 16">
@@ -629,6 +632,136 @@
             <a:xfrm>
               <a:off x="6484807" y="1412955"/>
               <a:ext cx="62640" cy="12600"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>461602</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>104625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>512002</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>104985</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="2" name="Freihand 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{327A6585-4B31-4225-A97E-E97841442423}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="6490927" y="1628625"/>
+            <a:ext cx="50400" cy="360"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="17" name="Freihand 16">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99DBE622-91D6-419B-B1A6-A87E82E9D18F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6484807" y="1412955"/>
+              <a:ext cx="62640" cy="12600"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>485618</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>54563</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>568778</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>136283</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="3" name="Freihand 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{008B3F99-3FA9-4E26-85ED-F15560C28F77}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7524593" y="1578563"/>
+            <a:ext cx="83160" cy="81720"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="5" name="Freihand 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1B923C7-17A5-470E-B6E7-A219965DFEC1}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7501830" y="1365300"/>
+              <a:ext cx="118800" cy="117360"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -670,6 +803,34 @@
 </inkml:ink>
 </file>
 
+<file path=xl/ink/ink10.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-12T15:42:07.209"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.1" units="cm"/>
+      <inkml:brushProperty name="height" value="0.1" units="cm"/>
+      <inkml:brushProperty name="color" value="#008C3A"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 113 9830,'1'11'364,"0"0"0,1 0 0,0-1 0,1 1 0,0-1 1,1 1-1,0-1 0,5 10 0,-9-20-335,1 1 0,-1-1 1,0 1-1,1-1 0,-1 1 1,1-1-1,-1 1 0,1-1 1,-1 1-1,1-1 0,-1 1 0,1-1 1,0 0-1,-1 1 0,1-1 1,-1 0-1,1 1 0,0-1 1,-1 0-1,1 0 0,0 0 0,0 0 1,-1 0-1,1 0 0,0 0 1,-1 0-1,1 0 0,1 0 1,21-12 25,16-27-449,-37 36 427,-1 2-46,17-19-100,0 0 1,-2-1 0,-1-1-1,0 0 1,12-28 0,-22 41 250,-1 2-101</inkml:trace>
+</inkml:ink>
+</file>
+
 <file path=xl/ink/ink2.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -853,6 +1014,33 @@
         </inkml:channelProperties>
       </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2026-03-12T10:36:20.134"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 0 24575,'2'0'0,"3"0"0,4 0 0,1 0 0,2 0 0,1 0 0,1 0 0,-1 0 0,1 0 0,2 0 0,1 0 0,-3 0-8191</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink9.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-12T15:41:58.817"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.035" units="cm"/>
@@ -1180,7 +1368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32591C64-F459-4437-AAEE-14859C7DF2EF}">
-  <dimension ref="F4:H10"/>
+  <dimension ref="F4:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="33.28515625" bestFit="1" customWidth="1"/>
@@ -1224,15 +1412,22 @@
     </row>
     <row r="9" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
     </row>
     <row r="10" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>